<commit_message>
Implementation except PFR Recycle
</commit_message>
<xml_diff>
--- a/Data/Data_Scripts_Evaluation/Calculation.xlsx
+++ b/Data/Data_Scripts_Evaluation/Calculation.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tuanaoyuncu/Documents/GitHub/nRTD/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tuanaoyuncu/Documents/GitHub/nRTD/Data/Data_Scripts_Evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B84C435F-F790-6A44-9928-65DA6E562E59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A85E444-0AF7-414F-ACF0-F8564AB813A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16280" xr2:uid="{24048C4F-BF72-8947-858C-9A2227B38C89}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="660" windowWidth="28800" windowHeight="16280" activeTab="1" xr2:uid="{24048C4F-BF72-8947-858C-9A2227B38C89}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Laminar" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="solver_adj" localSheetId="0" hidden="1">Sheet1!$E$10</definedName>
@@ -63,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="8">
   <si>
     <t>DeltaT_E</t>
   </si>
@@ -882,4 +883,71 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6391877-51E4-D242-9782-E0B87465A1CE}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1">
+        <v>30</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="1">
+        <f>A4</f>
+        <v>166.33333333333331</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <f>B1-B2</f>
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1">
+        <f>E1-1-E2</f>
+        <v>332.66666666666669</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <f>((E1-1)*(1/(1+B2/B3)))</f>
+        <v>166.33333333333331</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Laminar Flow model investigation is done
</commit_message>
<xml_diff>
--- a/Data/Data_Scripts_Evaluation/Calculation.xlsx
+++ b/Data/Data_Scripts_Evaluation/Calculation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tuanaoyuncu/Documents/GitHub/nRTD/Data/Data_Scripts_Evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CD156EE-1B1B-4D43-8E57-E7A972E0FFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{263B4544-9199-4048-94D6-FABD3432684B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16280" activeTab="1" xr2:uid="{24048C4F-BF72-8947-858C-9A2227B38C89}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16280" activeTab="1" xr2:uid="{24048C4F-BF72-8947-858C-9A2227B38C89}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="9">
   <si>
     <t>DeltaT_E</t>
   </si>
@@ -89,6 +89,9 @@
   <si>
     <t>N_E</t>
   </si>
+  <si>
+    <t>LAMINAR</t>
+  </si>
 </sst>
 </file>
 
@@ -110,12 +113,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -130,11 +145,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -887,7 +904,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6391877-51E4-D242-9782-E0B87465A1CE}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -895,7 +912,7 @@
         <v>1</v>
       </c>
       <c r="B1">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="C1" t="s">
         <v>3</v>
@@ -919,7 +936,7 @@
       </c>
       <c r="E2" s="1">
         <f>A4</f>
-        <v>277.22222222222223</v>
+        <v>399.20000000000005</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -928,7 +945,7 @@
       </c>
       <c r="B3">
         <f>B1-B2</f>
-        <v>25</v>
+        <v>80</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
@@ -938,14 +955,282 @@
       </c>
       <c r="E3" s="1">
         <f>E1-1-E2</f>
-        <v>221.77777777777777</v>
+        <v>99.799999999999955</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <f>((E1-1)*(1/(1+B2/B3)))</f>
-        <v>277.22222222222223</v>
-      </c>
+        <v>399.20000000000005</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="5">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>60</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9">
+        <v>30</v>
+      </c>
+      <c r="D9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="1">
+        <f>A11</f>
+        <v>249.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10">
+        <f>B8-B9</f>
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="1">
+        <f>E8-A11-1</f>
+        <v>249.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <f>((E8-1)*(1/(1+B9/B10)))</f>
+        <v>249.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="5">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" s="2">
+        <v>60</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" s="2">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" s="2">
+        <v>30</v>
+      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" s="3">
+        <f>A17</f>
+        <v>199.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="2">
+        <f>B14-B15</f>
+        <v>30</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="3">
+        <f>E14-A17-2</f>
+        <v>198.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="3">
+        <f>((E14-1)*(1/(1+B15/B16)))</f>
+        <v>199.5</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="5">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" s="2">
+        <v>60</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E20" s="2">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B21" s="2">
+        <v>30</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E21" s="3">
+        <f>A23</f>
+        <v>149.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" s="2">
+        <f>B20-B21</f>
+        <v>30</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E22" s="3">
+        <f>E20-A23-2</f>
+        <v>148.5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="3">
+        <f>((E20-1)*(1/(1+B21/B22)))</f>
+        <v>149.5</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="5">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="2">
+        <v>60</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E26" s="2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B27" s="2">
+        <v>30</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E27" s="3">
+        <f>A29</f>
+        <v>49.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B28" s="2">
+        <f>B26-B27</f>
+        <v>30</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E28" s="3">
+        <f>E26-A29-2</f>
+        <v>48.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="3">
+        <f>((E26-1)*(1/(1+B27/B28)))</f>
+        <v>49.5</v>
+      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Noisy and 2nd layer work
</commit_message>
<xml_diff>
--- a/Data/Data_Scripts_Evaluation/Calculation.xlsx
+++ b/Data/Data_Scripts_Evaluation/Calculation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tuanaoyuncu/Documents/GitHub/nRTD/Data/Data_Scripts_Evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8435B800-FE6D-4349-ACB2-45F6D7A8339F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07BC0B8E-4DEA-1C45-A508-5174B3207054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12980" yWindow="500" windowWidth="28800" windowHeight="16460" activeTab="1" xr2:uid="{24048C4F-BF72-8947-858C-9A2227B38C89}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16400" activeTab="1" xr2:uid="{24048C4F-BF72-8947-858C-9A2227B38C89}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="13">
   <si>
     <t>DeltaT_E</t>
   </si>
@@ -923,7 +923,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6391877-51E4-D242-9782-E0B87465A1CE}">
-  <dimension ref="A1:AC35"/>
+  <dimension ref="A1:AC52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="6" max="6" width="10.83203125" style="6"/>
@@ -1307,6 +1307,9 @@
       <c r="M14" s="5">
         <v>300</v>
       </c>
+      <c r="S14">
+        <v>200</v>
+      </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
@@ -1353,6 +1356,21 @@
       <c r="Q15">
         <v>300</v>
       </c>
+      <c r="S15" t="s">
+        <v>1</v>
+      </c>
+      <c r="T15">
+        <v>45</v>
+      </c>
+      <c r="U15" t="s">
+        <v>3</v>
+      </c>
+      <c r="V15" t="s">
+        <v>5</v>
+      </c>
+      <c r="W15">
+        <v>500</v>
+      </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
@@ -1398,8 +1416,21 @@
         <f>M18</f>
         <v>166.11111111111111</v>
       </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="S16" t="s">
+        <v>2</v>
+      </c>
+      <c r="T16">
+        <v>25</v>
+      </c>
+      <c r="V16" t="s">
+        <v>6</v>
+      </c>
+      <c r="W16" s="1">
+        <f>S18</f>
+        <v>221.77777777777777</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <f>((E14-1)*(1/(1+B15/B16)))</f>
         <v>199.5</v>
@@ -1442,8 +1473,25 @@
         <f>Q15-M18-1</f>
         <v>132.88888888888889</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="S17" t="s">
+        <v>0</v>
+      </c>
+      <c r="T17">
+        <f>T15-T16</f>
+        <v>20</v>
+      </c>
+      <c r="U17" t="s">
+        <v>4</v>
+      </c>
+      <c r="V17" t="s">
+        <v>7</v>
+      </c>
+      <c r="W17" s="1">
+        <f>W15-S18-1</f>
+        <v>277.22222222222223</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="G18" s="1">
         <f>((K15-1)*(1/(1+H16/H17)))</f>
         <v>29.7</v>
@@ -1452,13 +1500,17 @@
         <f>((Q15-1)*(1/(1+N16/N17)))</f>
         <v>166.11111111111111</v>
       </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="S18" s="1">
+        <f>((W15-1)*(1/(1+T16/T17)))</f>
+        <v>221.77777777777777</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A19" s="5">
         <v>300</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>1</v>
       </c>
@@ -1481,7 +1533,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>2</v>
       </c>
@@ -1526,8 +1578,11 @@
       <c r="Q21">
         <v>200</v>
       </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="S21">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>0</v>
       </c>
@@ -1571,8 +1626,23 @@
         <f>M24</f>
         <v>110.55555555555556</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="S22" t="s">
+        <v>1</v>
+      </c>
+      <c r="T22">
+        <v>45</v>
+      </c>
+      <c r="U22" t="s">
+        <v>3</v>
+      </c>
+      <c r="V22" t="s">
+        <v>5</v>
+      </c>
+      <c r="W22">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <f>((E20-1)*(1/(1+B21/B22)))</f>
         <v>149.5</v>
@@ -1615,8 +1685,21 @@
         <f>Q21-M24-1</f>
         <v>88.444444444444443</v>
       </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="S23" t="s">
+        <v>2</v>
+      </c>
+      <c r="T23">
+        <v>25</v>
+      </c>
+      <c r="V23" t="s">
+        <v>6</v>
+      </c>
+      <c r="W23" s="1">
+        <f>S25</f>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
       <c r="G24" s="1">
         <f>((K21-1)*(1/(1+H22/H23)))</f>
         <v>149.5</v>
@@ -1625,16 +1708,37 @@
         <f>((Q21-1)*(1/(1+N22/N23)))</f>
         <v>110.55555555555556</v>
       </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="S24" t="s">
+        <v>0</v>
+      </c>
+      <c r="T24">
+        <f>T22-T23</f>
+        <v>20</v>
+      </c>
+      <c r="U24" t="s">
+        <v>4</v>
+      </c>
+      <c r="V24" t="s">
+        <v>7</v>
+      </c>
+      <c r="W24" s="1">
+        <f>W22-S25-1</f>
+        <v>185</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A25" s="5">
         <v>200</v>
       </c>
       <c r="G25">
         <v>200</v>
       </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="S25" s="1">
+        <f>((W22-1)*(1/(1+T23/T24)))</f>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>1</v>
       </c>
@@ -1666,7 +1770,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>2</v>
       </c>
@@ -1695,7 +1799,7 @@
         <v>99.5</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>0</v>
       </c>
@@ -1731,7 +1835,7 @@
         <v>98.5</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <f>((E26-1)*(1/(1+B27/B28)))</f>
         <v>99.5</v>
@@ -1745,7 +1849,7 @@
         <v>99.5</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" s="5">
         <v>200</v>
       </c>
@@ -1753,7 +1857,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>1</v>
       </c>
@@ -1864,6 +1968,204 @@
         <v>99.5</v>
       </c>
     </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A37" s="5">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B38" s="2">
+        <v>60</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E38" s="2">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B39" s="2">
+        <v>30</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E39" s="3">
+        <f>A41</f>
+        <v>166.5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" s="2">
+        <f>B38-B39</f>
+        <v>30</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E40" s="3">
+        <f>E38-A41-2</f>
+        <v>165.5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A41" s="3">
+        <f>((E38-1)*(1/(1+B39/B40)))</f>
+        <v>166.5</v>
+      </c>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B44" s="2">
+        <v>60</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E44" s="2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B45" s="2">
+        <v>30</v>
+      </c>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E45" s="3">
+        <f>A47</f>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B46" s="2">
+        <f>B44-B45</f>
+        <v>30</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E46" s="3">
+        <f>E44-A47-2</f>
+        <v>82</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A47" s="3">
+        <f>((E44-1)*(1/(1+B45/B46)))</f>
+        <v>83</v>
+      </c>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B49" s="2">
+        <v>60</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E49" s="2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B50" s="2">
+        <v>30</v>
+      </c>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E50" s="3">
+        <f>A52</f>
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B51" s="2">
+        <f>B49-B50</f>
+        <v>30</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E51" s="3">
+        <f>E49-A52-2</f>
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" s="3">
+        <f>((E49-1)*(1/(1+B50/B51)))</f>
+        <v>41.5</v>
+      </c>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>